<commit_message>
Price list: one spelling per pack size for the oz bags
Justin, 2026-09-14: Java said 11oz foil bag where its siblings said 11oz bag.
All 25 eleven-ounce chicory bags now read 11oz bag, and the same collapse is
applied to the 10oz, 7.9oz, 3.53oz, 3.95oz, 4.76oz and 8.9oz families.
39 items, 36 distinct size strings down to 32.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopify-price-list.xlsx
+++ b/shopify-price-list.xlsx
@@ -4334,7 +4334,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E93" s="2" t="n">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E96" s="2" t="n">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>10oz</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E98" s="2" t="n">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
@@ -4884,7 +4884,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E105" s="2" t="n">
@@ -5021,7 +5021,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E108" s="2" t="n">
@@ -5387,7 +5387,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E116" s="2" t="n">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E123" s="2" t="n">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E141" s="2" t="n">
@@ -6718,7 +6718,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E145" s="2" t="n">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E154" s="2" t="n">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>10oz</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E158" s="2" t="n">
@@ -7362,7 +7362,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E159" s="2" t="n">
@@ -7454,7 +7454,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E161" s="2" t="n">
@@ -7591,7 +7591,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E164" s="2" t="n">
@@ -7683,7 +7683,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E166" s="2" t="n">
@@ -8280,7 +8280,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E179" s="2" t="n">
@@ -8372,7 +8372,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E181" s="2" t="n">
@@ -8556,7 +8556,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E185" s="2" t="n">
@@ -8740,7 +8740,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E189" s="2" t="n">
@@ -8832,7 +8832,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E191" s="2" t="n">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E200" s="2" t="n">
@@ -9380,7 +9380,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E203" s="2" t="n">
@@ -13022,7 +13022,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E281" s="2" t="n">
@@ -13069,7 +13069,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E282" s="2" t="n">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E283" s="2" t="n">
@@ -13163,7 +13163,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E284" s="2" t="n">
@@ -13210,7 +13210,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E285" s="2" t="n">
@@ -13257,7 +13257,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>3.95oz foil bag</t>
+          <t>3.95oz bag</t>
         </is>
       </c>
       <c r="E286" s="2" t="n">
@@ -13304,7 +13304,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E287" s="2" t="n">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E288" s="2" t="n">
@@ -13398,7 +13398,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E289" s="2" t="n">
@@ -13445,7 +13445,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E290" s="2" t="n">
@@ -13492,7 +13492,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E291" s="2" t="n">
@@ -13539,7 +13539,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E292" s="2" t="n">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>8.9oz foil bag</t>
+          <t>8.9oz bag</t>
         </is>
       </c>
       <c r="E293" s="2" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>4.76oz foil bag</t>
+          <t>4.76oz bag</t>
         </is>
       </c>
       <c r="E294" s="2" t="n">
@@ -15071,7 +15071,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -15118,7 +15118,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -15165,7 +15165,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -15212,7 +15212,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.53oz foil bag</t>
+          <t>3.53oz bag</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -15306,7 +15306,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.95oz foil bag</t>
+          <t>3.95oz bag</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -15973,7 +15973,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.76oz foil bag</t>
+          <t>4.76oz bag</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -16150,7 +16150,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -16379,7 +16379,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10oz</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -16426,7 +16426,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -16700,7 +16700,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -16837,7 +16837,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -17203,7 +17203,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -17524,7 +17524,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E33" s="2" t="n">
@@ -18350,7 +18350,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
@@ -18534,7 +18534,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
@@ -18947,7 +18947,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
@@ -19131,7 +19131,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10oz</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E68" s="2" t="n">
@@ -19178,7 +19178,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E69" s="2" t="n">
@@ -19270,7 +19270,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
@@ -19407,7 +19407,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
@@ -19499,7 +19499,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
@@ -20096,7 +20096,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E89" s="2" t="n">
@@ -20188,7 +20188,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E91" s="2" t="n">
@@ -20372,7 +20372,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E95" s="2" t="n">
@@ -20556,7 +20556,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>11oz</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E99" s="2" t="n">
@@ -20648,7 +20648,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E101" s="2" t="n">
@@ -21059,7 +21059,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>10oz foil bag</t>
+          <t>10oz bag</t>
         </is>
       </c>
       <c r="E110" s="2" t="n">
@@ -21196,7 +21196,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>11oz foil bag</t>
+          <t>11oz bag</t>
         </is>
       </c>
       <c r="E113" s="2" t="n">
@@ -30120,7 +30120,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -30167,7 +30167,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -30214,7 +30214,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -30261,7 +30261,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -30308,7 +30308,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -30355,7 +30355,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>7.9oz foil bag</t>
+          <t>7.9oz bag</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -30400,7 +30400,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8.9oz foil bag</t>
+          <t>8.9oz bag</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">

</xml_diff>

<commit_message>
Price list: tea counts collapse to 25ct box, 10ct box, 12ct box
Justin picked the wording. 45 more items normalised - 25ct tea bag box,
10ct tea bag box and 12ct tea bag box lose the content descriptor, matching
the 11oz bag pattern. Size vocabulary is now 23 distinct values, down from 36.

The 18 rows still showing a bare count (50ct, 25ct, 6ct) take their size from
the Amazon channel because our own record has none; a container word there
would be invented, so they stay bare and the gap stays visible.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopify-price-list.xlsx
+++ b/shopify-price-list.xlsx
@@ -2343,7 +2343,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>48 ct</t>
+          <t>48ct</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
@@ -3994,7 +3994,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>24 ct</t>
+          <t>24ct</t>
         </is>
       </c>
       <c r="E85" s="2" t="n">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E206" s="2" t="n">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E209" s="2" t="n">
@@ -9754,7 +9754,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E211" s="2" t="n">
@@ -9801,7 +9801,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E212" s="2" t="n">
@@ -9942,7 +9942,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E215" s="2" t="n">
@@ -9989,7 +9989,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E216" s="2" t="n">
@@ -10079,7 +10079,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E218" s="2" t="n">
@@ -10126,7 +10126,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E219" s="2" t="n">
@@ -10173,7 +10173,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E220" s="2" t="n">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E221" s="2" t="n">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E222" s="2" t="n">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E223" s="2" t="n">
@@ -10361,7 +10361,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E224" s="2" t="n">
@@ -10408,7 +10408,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E225" s="2" t="n">
@@ -10455,7 +10455,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E226" s="2" t="n">
@@ -10502,7 +10502,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E227" s="2" t="n">
@@ -10549,7 +10549,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E228" s="2" t="n">
@@ -10643,7 +10643,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>10 ct</t>
+          <t>10ct</t>
         </is>
       </c>
       <c r="E230" s="2" t="n">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>10 ct</t>
+          <t>10ct</t>
         </is>
       </c>
       <c r="E232" s="2" t="n">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E234" s="2" t="n">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E235" s="2" t="n">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E236" s="2" t="n">
@@ -11019,7 +11019,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E238" s="2" t="n">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E239" s="2" t="n">
@@ -11113,7 +11113,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E240" s="2" t="n">
@@ -11254,7 +11254,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E243" s="2" t="n">
@@ -11301,7 +11301,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E244" s="2" t="n">
@@ -11348,7 +11348,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E245" s="2" t="n">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E246" s="2" t="n">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E247" s="2" t="n">
@@ -11489,7 +11489,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E248" s="2" t="n">
@@ -11536,7 +11536,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E249" s="2" t="n">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E250" s="2" t="n">
@@ -11630,7 +11630,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E251" s="2" t="n">
@@ -11677,7 +11677,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E252" s="2" t="n">
@@ -11724,7 +11724,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E253" s="2" t="n">
@@ -11818,7 +11818,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E255" s="2" t="n">
@@ -11912,7 +11912,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E257" s="2" t="n">
@@ -12006,7 +12006,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E259" s="2" t="n">
@@ -12053,7 +12053,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E260" s="2" t="n">
@@ -12100,7 +12100,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E261" s="2" t="n">
@@ -12143,7 +12143,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E262" s="2" t="n">
@@ -12190,7 +12190,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E263" s="2" t="n">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E264" s="2" t="n">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E265" s="2" t="n">
@@ -12421,7 +12421,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E268" s="2" t="n">
@@ -12468,7 +12468,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E269" s="2" t="n">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E270" s="2" t="n">
@@ -12740,7 +12740,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E275" s="2" t="n">
@@ -12787,7 +12787,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E276" s="2" t="n">
@@ -12834,7 +12834,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E277" s="2" t="n">
@@ -12881,7 +12881,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E278" s="2" t="n">
@@ -12928,7 +12928,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E279" s="2" t="n">
@@ -12975,7 +12975,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E280" s="2" t="n">
@@ -13805,7 +13805,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E298" s="2" t="n">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>6 ct</t>
+          <t>6ct</t>
         </is>
       </c>
       <c r="E299" s="2" t="n">
@@ -13899,7 +13899,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E300" s="2" t="n">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E302" s="2" t="n">
@@ -14079,7 +14079,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E304" s="2" t="n">
@@ -14126,7 +14126,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>6 ct</t>
+          <t>6ct</t>
         </is>
       </c>
       <c r="E305" s="2" t="n">
@@ -14216,7 +14216,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>12 ct</t>
+          <t>12ct</t>
         </is>
       </c>
       <c r="E307" s="2" t="n">
@@ -21420,7 +21420,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -21561,7 +21561,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -21655,7 +21655,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -21702,7 +21702,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -21843,7 +21843,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -21890,7 +21890,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -21980,7 +21980,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -22027,7 +22027,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -22074,7 +22074,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -22121,7 +22121,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -22168,7 +22168,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -22215,7 +22215,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
@@ -22262,7 +22262,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -22309,7 +22309,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
@@ -22356,7 +22356,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -22403,7 +22403,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
@@ -22450,7 +22450,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
@@ -22544,7 +22544,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10 ct</t>
+          <t>10ct</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -22638,7 +22638,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>10 ct</t>
+          <t>10ct</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
@@ -22732,7 +22732,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E30" s="2" t="n">
@@ -22779,7 +22779,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
@@ -22826,7 +22826,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
@@ -22920,7 +22920,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E34" s="2" t="n">
@@ -22967,7 +22967,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E35" s="2" t="n">
@@ -23014,7 +23014,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
@@ -23155,7 +23155,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E39" s="2" t="n">
@@ -23202,7 +23202,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E40" s="2" t="n">
@@ -23249,7 +23249,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E41" s="2" t="n">
@@ -23296,7 +23296,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E42" s="2" t="n">
@@ -23343,7 +23343,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
@@ -23390,7 +23390,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E44" s="2" t="n">
@@ -23437,7 +23437,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
@@ -23484,7 +23484,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E46" s="2" t="n">
@@ -23531,7 +23531,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E47" s="2" t="n">
@@ -23578,7 +23578,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E48" s="2" t="n">
@@ -23625,7 +23625,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
@@ -23719,7 +23719,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E53" s="2" t="n">
@@ -23907,7 +23907,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E55" s="2" t="n">
@@ -23954,7 +23954,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E56" s="2" t="n">
@@ -24001,7 +24001,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E57" s="2" t="n">
@@ -24044,7 +24044,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E58" s="2" t="n">
@@ -24091,7 +24091,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E59" s="2" t="n">
@@ -24138,7 +24138,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E60" s="2" t="n">
@@ -24185,7 +24185,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>25 ct</t>
+          <t>25ct</t>
         </is>
       </c>
       <c r="E61" s="2" t="n">
@@ -24322,7 +24322,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E64" s="2" t="n">
@@ -24369,7 +24369,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
@@ -24416,7 +24416,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E66" s="2" t="n">
@@ -24641,7 +24641,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
@@ -24688,7 +24688,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E72" s="2" t="n">
@@ -24735,7 +24735,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E73" s="2" t="n">
@@ -24782,7 +24782,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>10ct tea bag box</t>
+          <t>10ct box</t>
         </is>
       </c>
       <c r="E74" s="2" t="n">
@@ -24829,7 +24829,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>25ct tea bag box</t>
+          <t>25ct box</t>
         </is>
       </c>
       <c r="E75" s="2" t="n">
@@ -24876,7 +24876,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>50 ct</t>
+          <t>50ct</t>
         </is>
       </c>
       <c r="E76" s="2" t="n">
@@ -25758,7 +25758,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>48 ct</t>
+          <t>48ct</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
@@ -27187,7 +27187,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -27234,7 +27234,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6 ct</t>
+          <t>6ct</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -27281,7 +27281,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -27371,7 +27371,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -27461,7 +27461,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>12ct tea bag box</t>
+          <t>12ct box</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -27508,7 +27508,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6 ct</t>
+          <t>6ct</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -27598,7 +27598,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>12 ct</t>
+          <t>12ct</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -29311,7 +29311,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>24 ct</t>
+          <t>24ct</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">

</xml_diff>

<commit_message>
Retail price list: publish a new-prices edition alongside the current one
Two trade-layout downloads on the page - one at the prices live on the site
today, one carrying the approved increase. The second prints "Effective the
approved increase (not yet live)" on its own date line so a copy cannot be
mistaken for a live list.

Both regenerate whenever the page does.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopify-price-list.xlsx
+++ b/shopify-price-list.xlsx
@@ -1963,7 +1963,11 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="B37" t="inlineStr">
         <is>
           <t>Fall Box - Herbal Coffee</t>
@@ -22426,7 +22430,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>Fall Box - Herbal Coffee</t>

</xml_diff>

<commit_message>
10ct teas held at the 9/15/26 MAP; fix plan selection picking a stale file
Justin, on Galens advice: drop the 10ct back rather than raise it, so iHerb
cannot undercut our own site. 15 ten-count rows removed from the increase;
their price and compare-at stay as they are. Plan 77 -> 62 rows.

Also fixed a real bug: the report chose its plan with sorted(glob())[-1], which
picked FINAL-TIDY over the newer FINAL-NO10CT because T sorts after N. The
export was publishing superseded prices from a file that had been replaced.
Plan selection now reads the internal generated timestamp - a filename is not
a clock.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopify-price-list.xlsx
+++ b/shopify-price-list.xlsx
@@ -8488,16 +8488,14 @@
         <v>8.99</v>
       </c>
       <c r="F184" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G184" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G184" s="3" t="n"/>
       <c r="H184" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I184" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
@@ -8672,16 +8670,14 @@
         <v>9.99</v>
       </c>
       <c r="F188" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G188" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G188" s="3" t="n"/>
       <c r="H188" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
@@ -8856,11 +8852,9 @@
         <v>9.99</v>
       </c>
       <c r="F192" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G192" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G192" s="3" t="n"/>
       <c r="H192" s="2" t="n"/>
       <c r="I192" s="2" t="n"/>
       <c r="J192" t="inlineStr">
@@ -8944,16 +8938,14 @@
         <v>9.99</v>
       </c>
       <c r="F194" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G194" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G194" s="3" t="n"/>
       <c r="H194" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J194" t="inlineStr">
         <is>
@@ -9177,16 +9169,14 @@
         <v>9.99</v>
       </c>
       <c r="F199" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G199" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G199" s="3" t="n"/>
       <c r="H199" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J199" t="inlineStr">
         <is>
@@ -9723,16 +9713,14 @@
         <v>10.99</v>
       </c>
       <c r="F211" s="2" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="G211" s="3" t="n">
-        <v>9.1</v>
-      </c>
+        <v>10.99</v>
+      </c>
+      <c r="G211" s="3" t="n"/>
       <c r="H211" s="2" t="n">
         <v>11.99</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>12.99</v>
+        <v>11.99</v>
       </c>
       <c r="J211" t="inlineStr">
         <is>
@@ -10093,16 +10081,14 @@
         <v>8.99</v>
       </c>
       <c r="F219" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G219" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G219" s="3" t="n"/>
       <c r="H219" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J219" t="inlineStr">
         <is>
@@ -10279,16 +10265,14 @@
         <v>8.99</v>
       </c>
       <c r="F223" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G223" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G223" s="3" t="n"/>
       <c r="H223" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J223" t="inlineStr">
         <is>
@@ -10416,16 +10400,14 @@
         <v>9.99</v>
       </c>
       <c r="F226" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G226" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G226" s="3" t="n"/>
       <c r="H226" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J226" t="inlineStr">
         <is>
@@ -10510,16 +10492,14 @@
         <v>8.99</v>
       </c>
       <c r="F228" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G228" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G228" s="3" t="n"/>
       <c r="H228" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J228" t="inlineStr">
         <is>
@@ -10737,11 +10717,9 @@
         <v>10.49</v>
       </c>
       <c r="F233" s="2" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="G233" s="3" t="n">
-        <v>14.3</v>
-      </c>
+        <v>10.49</v>
+      </c>
+      <c r="G233" s="3" t="n"/>
       <c r="H233" s="2" t="n"/>
       <c r="I233" s="2" t="n"/>
       <c r="J233" t="inlineStr">
@@ -11009,16 +10987,14 @@
         <v>9.99</v>
       </c>
       <c r="F239" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G239" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G239" s="3" t="n"/>
       <c r="H239" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I239" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J239" t="inlineStr">
         <is>
@@ -11101,16 +11077,14 @@
         <v>8.99</v>
       </c>
       <c r="F241" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G241" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G241" s="3" t="n"/>
       <c r="H241" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I241" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J241" t="inlineStr">
         <is>
@@ -11322,16 +11296,14 @@
         <v>9.99</v>
       </c>
       <c r="F246" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G246" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G246" s="3" t="n"/>
       <c r="H246" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I246" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J246" t="inlineStr">
         <is>
@@ -11416,16 +11388,14 @@
         <v>8.99</v>
       </c>
       <c r="F248" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G248" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G248" s="3" t="n"/>
       <c r="H248" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I248" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J248" t="inlineStr">
         <is>
@@ -18913,16 +18883,14 @@
         <v>8.99</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G2" s="3" t="n"/>
       <c r="H2" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -19097,16 +19065,14 @@
         <v>9.99</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G6" s="3" t="n"/>
       <c r="H6" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -19281,11 +19247,9 @@
         <v>9.99</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G10" s="3" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
       <c r="J10" t="inlineStr">
@@ -19369,16 +19333,14 @@
         <v>9.99</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G12" s="3" t="n"/>
       <c r="H12" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -19602,16 +19564,14 @@
         <v>9.99</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G17" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G17" s="3" t="n"/>
       <c r="H17" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -20148,16 +20108,14 @@
         <v>10.99</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>9.1</v>
-      </c>
+        <v>10.99</v>
+      </c>
+      <c r="G29" s="3" t="n"/>
       <c r="H29" s="2" t="n">
         <v>11.99</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>12.99</v>
+        <v>11.99</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -20518,16 +20476,14 @@
         <v>8.99</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G37" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G37" s="3" t="n"/>
       <c r="H37" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -20704,16 +20660,14 @@
         <v>8.99</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G41" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G41" s="3" t="n"/>
       <c r="H41" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -20841,16 +20795,14 @@
         <v>9.99</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G44" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G44" s="3" t="n"/>
       <c r="H44" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -20935,16 +20887,14 @@
         <v>8.99</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G46" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G46" s="3" t="n"/>
       <c r="H46" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -21162,11 +21112,9 @@
         <v>10.49</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>11.99</v>
-      </c>
-      <c r="G51" s="3" t="n">
-        <v>14.3</v>
-      </c>
+        <v>10.49</v>
+      </c>
+      <c r="G51" s="3" t="n"/>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="n"/>
       <c r="J51" t="inlineStr">
@@ -21434,16 +21382,14 @@
         <v>9.99</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G57" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G57" s="3" t="n"/>
       <c r="H57" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -21526,16 +21472,14 @@
         <v>8.99</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G59" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G59" s="3" t="n"/>
       <c r="H59" s="2" t="n">
         <v>9.99</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>10.99</v>
+        <v>9.99</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -21747,16 +21691,14 @@
         <v>9.99</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>10.99</v>
-      </c>
-      <c r="G64" s="3" t="n">
-        <v>10</v>
-      </c>
+        <v>9.99</v>
+      </c>
+      <c r="G64" s="3" t="n"/>
       <c r="H64" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -21841,16 +21783,14 @@
         <v>8.99</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="G66" s="3" t="n">
-        <v>11.1</v>
-      </c>
+        <v>8.99</v>
+      </c>
+      <c r="G66" s="3" t="n"/>
       <c r="H66" s="2" t="n">
         <v>10.99</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>11.99</v>
+        <v>10.99</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Price list: increase applied 2026-09-18; retire the pending 'new prices' edition
The 62-row DTC increase landed and was verified live, so 'current prices' IS
the new price set. A second trade document marked 'not yet live' could now only
contradict it - and a forwarded copy would state something false to a trade
customer. Button, build and publish removed; build_retail_price_list keeps its
--prices pending switch for the next increase.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopify-price-list.xlsx
+++ b/shopify-price-list.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -2402,16 +2402,14 @@
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" s="2" t="n">
-        <v>34.99</v>
+        <v>37.99</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>37.99</v>
       </c>
-      <c r="H46" s="3" t="n">
-        <v>8.6</v>
-      </c>
+      <c r="H46" s="3" t="n"/>
       <c r="I46" s="2" t="n">
-        <v>38.49</v>
+        <v>41.99</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>41.99</v>
@@ -4092,16 +4090,14 @@
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" s="2" t="n">
-        <v>24.99</v>
+        <v>29.99</v>
       </c>
       <c r="G85" s="2" t="n">
         <v>29.99</v>
       </c>
-      <c r="H85" s="3" t="n">
-        <v>20</v>
-      </c>
+      <c r="H85" s="3" t="n"/>
       <c r="I85" s="2" t="n">
-        <v>27.49</v>
+        <v>32.99</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>32.99</v>
@@ -4440,16 +4436,14 @@
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G93" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H93" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H93" s="3" t="n"/>
       <c r="I93" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>19.49</v>
@@ -4730,16 +4724,14 @@
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G99" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H99" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H99" s="3" t="n"/>
       <c r="I99" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>19.49</v>
@@ -5020,16 +5012,14 @@
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G105" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H105" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H105" s="3" t="n"/>
       <c r="I105" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>21.99</v>
@@ -5160,16 +5150,14 @@
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G108" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H108" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H108" s="3" t="n"/>
       <c r="I108" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>19.49</v>
@@ -5544,16 +5532,14 @@
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G116" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H116" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H116" s="3" t="n"/>
       <c r="I116" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>21.99</v>
@@ -5592,16 +5578,14 @@
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" s="2" t="n">
-        <v>31.99</v>
+        <v>34.99</v>
       </c>
       <c r="G117" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H117" s="3" t="n">
-        <v>9.4</v>
-      </c>
+      <c r="H117" s="3" t="n"/>
       <c r="I117" s="2" t="n">
-        <v>34.99</v>
+        <v>38.49</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>38.49</v>
@@ -5916,16 +5900,14 @@
       </c>
       <c r="E124" t="inlineStr"/>
       <c r="F124" s="2" t="n">
-        <v>31.99</v>
+        <v>34.99</v>
       </c>
       <c r="G124" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H124" s="3" t="n">
-        <v>9.4</v>
-      </c>
+      <c r="H124" s="3" t="n"/>
       <c r="I124" s="2" t="n">
-        <v>34.99</v>
+        <v>38.49</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>38.49</v>
@@ -6712,16 +6694,14 @@
       </c>
       <c r="E141" t="inlineStr"/>
       <c r="F141" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G141" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H141" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H141" s="3" t="n"/>
       <c r="I141" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J141" s="2" t="n">
         <v>23.99</v>
@@ -6806,16 +6786,14 @@
       </c>
       <c r="E143" t="inlineStr"/>
       <c r="F143" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G143" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H143" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H143" s="3" t="n"/>
       <c r="I143" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J143" s="2" t="n">
         <v>19.49</v>
@@ -6900,16 +6878,14 @@
       </c>
       <c r="E145" t="inlineStr"/>
       <c r="F145" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G145" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H145" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H145" s="3" t="n"/>
       <c r="I145" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J145" s="2" t="n">
         <v>19.49</v>
@@ -6948,16 +6924,14 @@
       </c>
       <c r="E146" t="inlineStr"/>
       <c r="F146" s="2" t="n">
-        <v>24.99</v>
+        <v>27.99</v>
       </c>
       <c r="G146" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H146" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="H146" s="3" t="n"/>
       <c r="I146" s="2" t="n">
-        <v>27.49</v>
+        <v>30.99</v>
       </c>
       <c r="J146" s="2" t="n">
         <v>30.99</v>
@@ -7322,16 +7296,14 @@
       </c>
       <c r="E154" t="inlineStr"/>
       <c r="F154" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G154" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H154" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H154" s="3" t="n"/>
       <c r="I154" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J154" s="2" t="n">
         <v>19.49</v>
@@ -7370,16 +7342,14 @@
       </c>
       <c r="E155" t="inlineStr"/>
       <c r="F155" s="2" t="n">
-        <v>21.99</v>
+        <v>27.99</v>
       </c>
       <c r="G155" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H155" s="3" t="n">
-        <v>27.3</v>
-      </c>
+      <c r="H155" s="3" t="n"/>
       <c r="I155" s="2" t="n">
-        <v>23.99</v>
+        <v>30.49</v>
       </c>
       <c r="J155" s="2" t="n">
         <v>30.49</v>
@@ -7556,16 +7526,14 @@
       </c>
       <c r="E159" t="inlineStr"/>
       <c r="F159" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G159" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H159" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H159" s="3" t="n"/>
       <c r="I159" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J159" s="2" t="n">
         <v>19.49</v>
@@ -7650,16 +7618,14 @@
       </c>
       <c r="E161" t="inlineStr"/>
       <c r="F161" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G161" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H161" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H161" s="3" t="n"/>
       <c r="I161" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J161" s="2" t="n">
         <v>19.49</v>
@@ -7790,16 +7756,14 @@
       </c>
       <c r="E164" t="inlineStr"/>
       <c r="F164" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G164" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H164" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H164" s="3" t="n"/>
       <c r="I164" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J164" s="2" t="n">
         <v>21.99</v>
@@ -7884,16 +7848,14 @@
       </c>
       <c r="E166" t="inlineStr"/>
       <c r="F166" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G166" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H166" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H166" s="3" t="n"/>
       <c r="I166" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J166" s="2" t="n">
         <v>19.49</v>
@@ -8512,16 +8474,14 @@
       </c>
       <c r="E179" t="inlineStr"/>
       <c r="F179" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G179" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H179" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H179" s="3" t="n"/>
       <c r="I179" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J179" s="2" t="n">
         <v>23.99</v>
@@ -8606,16 +8566,14 @@
       </c>
       <c r="E181" t="inlineStr"/>
       <c r="F181" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G181" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H181" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H181" s="3" t="n"/>
       <c r="I181" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J181" s="2" t="n">
         <v>19.49</v>
@@ -8654,16 +8612,14 @@
       </c>
       <c r="E182" t="inlineStr"/>
       <c r="F182" s="2" t="n">
-        <v>24.99</v>
+        <v>27.99</v>
       </c>
       <c r="G182" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H182" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="H182" s="3" t="n"/>
       <c r="I182" s="2" t="n">
-        <v>27.49</v>
+        <v>30.99</v>
       </c>
       <c r="J182" s="2" t="n">
         <v>30.99</v>
@@ -9496,16 +9452,14 @@
       </c>
       <c r="E200" t="inlineStr"/>
       <c r="F200" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G200" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H200" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H200" s="3" t="n"/>
       <c r="I200" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J200" s="2" t="n">
         <v>21.99</v>
@@ -9636,16 +9590,14 @@
       </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G203" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H203" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H203" s="3" t="n"/>
       <c r="I203" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J203" s="2" t="n">
         <v>19.49</v>
@@ -9684,16 +9636,14 @@
       </c>
       <c r="E204" t="inlineStr"/>
       <c r="F204" s="2" t="n">
-        <v>24.99</v>
+        <v>27.99</v>
       </c>
       <c r="G204" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H204" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="H204" s="3" t="n"/>
       <c r="I204" s="2" t="n">
-        <v>27.49</v>
+        <v>30.99</v>
       </c>
       <c r="J204" s="2" t="n">
         <v>30.99</v>
@@ -9916,16 +9866,14 @@
       </c>
       <c r="E209" t="inlineStr"/>
       <c r="F209" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G209" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H209" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H209" s="3" t="n"/>
       <c r="I209" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J209" s="2" t="n">
         <v>19.49</v>
@@ -10384,16 +10332,14 @@
       </c>
       <c r="E219" t="inlineStr"/>
       <c r="F219" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G219" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H219" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H219" s="3" t="n"/>
       <c r="I219" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J219" s="2" t="n">
         <v>21.99</v>
@@ -10432,16 +10378,14 @@
       </c>
       <c r="E220" t="inlineStr"/>
       <c r="F220" s="2" t="n">
-        <v>29.99</v>
+        <v>32.99</v>
       </c>
       <c r="G220" s="2" t="n">
         <v>32.99</v>
       </c>
-      <c r="H220" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H220" s="3" t="n"/>
       <c r="I220" s="2" t="n">
-        <v>32.99</v>
+        <v>36.49</v>
       </c>
       <c r="J220" s="2" t="n">
         <v>36.49</v>
@@ -10526,16 +10470,14 @@
       </c>
       <c r="E222" t="inlineStr"/>
       <c r="F222" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G222" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H222" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H222" s="3" t="n"/>
       <c r="I222" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J222" s="2" t="n">
         <v>21.99</v>
@@ -10666,16 +10608,14 @@
       </c>
       <c r="E225" t="inlineStr"/>
       <c r="F225" s="2" t="n">
-        <v>29.99</v>
+        <v>32.99</v>
       </c>
       <c r="G225" s="2" t="n">
         <v>32.99</v>
       </c>
-      <c r="H225" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H225" s="3" t="n"/>
       <c r="I225" s="2" t="n">
-        <v>32.99</v>
+        <v>36.49</v>
       </c>
       <c r="J225" s="2" t="n">
         <v>36.49</v>
@@ -11082,16 +11022,14 @@
       </c>
       <c r="E234" t="inlineStr"/>
       <c r="F234" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G234" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H234" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H234" s="3" t="n"/>
       <c r="I234" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J234" s="2" t="n">
         <v>21.99</v>
@@ -11222,16 +11160,14 @@
       </c>
       <c r="E237" t="inlineStr"/>
       <c r="F237" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G237" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H237" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H237" s="3" t="n"/>
       <c r="I237" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J237" s="2" t="n">
         <v>19.49</v>
@@ -11316,16 +11252,14 @@
       </c>
       <c r="E239" t="inlineStr"/>
       <c r="F239" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G239" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H239" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H239" s="3" t="n"/>
       <c r="I239" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J239" s="2" t="n">
         <v>19.49</v>
@@ -11364,16 +11298,14 @@
       </c>
       <c r="E240" t="inlineStr"/>
       <c r="F240" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G240" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H240" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H240" s="3" t="n"/>
       <c r="I240" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J240" s="2" t="n">
         <v>25.99</v>
@@ -11458,16 +11390,14 @@
       </c>
       <c r="E242" t="inlineStr"/>
       <c r="F242" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G242" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H242" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H242" s="3" t="n"/>
       <c r="I242" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J242" s="2" t="n">
         <v>19.49</v>
@@ -11598,16 +11528,14 @@
       </c>
       <c r="E245" t="inlineStr"/>
       <c r="F245" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G245" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H245" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H245" s="3" t="n"/>
       <c r="I245" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J245" s="2" t="n">
         <v>25.99</v>
@@ -11646,16 +11574,14 @@
       </c>
       <c r="E246" t="inlineStr"/>
       <c r="F246" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G246" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H246" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H246" s="3" t="n"/>
       <c r="I246" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J246" s="2" t="n">
         <v>21.99</v>
@@ -11878,16 +11804,14 @@
       </c>
       <c r="E251" t="inlineStr"/>
       <c r="F251" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G251" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H251" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H251" s="3" t="n"/>
       <c r="I251" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J251" s="2" t="n">
         <v>21.99</v>
@@ -12398,16 +12322,14 @@
       </c>
       <c r="E262" t="inlineStr"/>
       <c r="F262" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G262" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H262" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H262" s="3" t="n"/>
       <c r="I262" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J262" s="2" t="n">
         <v>23.99</v>
@@ -12446,16 +12368,14 @@
       </c>
       <c r="E263" t="inlineStr"/>
       <c r="F263" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G263" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H263" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H263" s="3" t="n"/>
       <c r="I263" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J263" s="2" t="n">
         <v>19.49</v>
@@ -12494,16 +12414,14 @@
       </c>
       <c r="E264" t="inlineStr"/>
       <c r="F264" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G264" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H264" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H264" s="3" t="n"/>
       <c r="I264" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J264" s="2" t="n">
         <v>25.99</v>
@@ -13094,16 +13012,14 @@
       </c>
       <c r="E277" t="inlineStr"/>
       <c r="F277" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G277" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H277" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H277" s="3" t="n"/>
       <c r="I277" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J277" s="2" t="n">
         <v>21.99</v>
@@ -13188,16 +13104,14 @@
       </c>
       <c r="E279" t="inlineStr"/>
       <c r="F279" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G279" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H279" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H279" s="3" t="n"/>
       <c r="I279" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J279" s="2" t="n">
         <v>19.49</v>
@@ -13236,16 +13150,14 @@
       </c>
       <c r="E280" t="inlineStr"/>
       <c r="F280" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G280" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H280" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H280" s="3" t="n"/>
       <c r="I280" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J280" s="2" t="n">
         <v>25.99</v>
@@ -13284,16 +13196,14 @@
       </c>
       <c r="E281" t="inlineStr"/>
       <c r="F281" s="2" t="n">
-        <v>24.99</v>
+        <v>29.99</v>
       </c>
       <c r="G281" s="2" t="n">
         <v>29.99</v>
       </c>
-      <c r="H281" s="3" t="n">
-        <v>20</v>
-      </c>
+      <c r="H281" s="3" t="n"/>
       <c r="I281" s="2" t="n">
-        <v>27.49</v>
+        <v>32.99</v>
       </c>
       <c r="J281" s="2" t="n">
         <v>32.99</v>
@@ -13332,16 +13242,14 @@
       </c>
       <c r="E282" t="inlineStr"/>
       <c r="F282" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G282" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H282" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H282" s="3" t="n"/>
       <c r="I282" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J282" s="2" t="n">
         <v>18.49</v>
@@ -13380,16 +13288,14 @@
       </c>
       <c r="E283" t="inlineStr"/>
       <c r="F283" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G283" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H283" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H283" s="3" t="n"/>
       <c r="I283" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J283" s="2" t="n">
         <v>18.49</v>
@@ -13428,16 +13334,14 @@
       </c>
       <c r="E284" t="inlineStr"/>
       <c r="F284" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G284" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H284" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H284" s="3" t="n"/>
       <c r="I284" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J284" s="2" t="n">
         <v>18.49</v>
@@ -13476,16 +13380,14 @@
       </c>
       <c r="E285" t="inlineStr"/>
       <c r="F285" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G285" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H285" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H285" s="3" t="n"/>
       <c r="I285" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J285" s="2" t="n">
         <v>18.49</v>
@@ -13524,16 +13426,14 @@
       </c>
       <c r="E286" t="inlineStr"/>
       <c r="F286" s="2" t="n">
-        <v>19.99</v>
+        <v>22.99</v>
       </c>
       <c r="G286" s="2" t="n">
         <v>22.99</v>
       </c>
-      <c r="H286" s="3" t="n">
-        <v>15</v>
-      </c>
+      <c r="H286" s="3" t="n"/>
       <c r="I286" s="2" t="n">
-        <v>21.99</v>
+        <v>25.49</v>
       </c>
       <c r="J286" s="2" t="n">
         <v>25.49</v>
@@ -13572,16 +13472,14 @@
       </c>
       <c r="E287" t="inlineStr"/>
       <c r="F287" s="2" t="n">
-        <v>22.99</v>
+        <v>24.99</v>
       </c>
       <c r="G287" s="2" t="n">
         <v>24.99</v>
       </c>
-      <c r="H287" s="3" t="n">
-        <v>8.699999999999999</v>
-      </c>
+      <c r="H287" s="3" t="n"/>
       <c r="I287" s="2" t="n">
-        <v>25.49</v>
+        <v>27.49</v>
       </c>
       <c r="J287" s="2" t="n">
         <v>27.49</v>
@@ -13620,16 +13518,14 @@
       </c>
       <c r="E288" t="inlineStr"/>
       <c r="F288" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G288" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H288" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H288" s="3" t="n"/>
       <c r="I288" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J288" s="2" t="n">
         <v>23.99</v>
@@ -13668,16 +13564,14 @@
       </c>
       <c r="E289" t="inlineStr"/>
       <c r="F289" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G289" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H289" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H289" s="3" t="n"/>
       <c r="I289" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J289" s="2" t="n">
         <v>23.99</v>
@@ -13716,16 +13610,14 @@
       </c>
       <c r="E290" t="inlineStr"/>
       <c r="F290" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G290" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H290" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H290" s="3" t="n"/>
       <c r="I290" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J290" s="2" t="n">
         <v>23.99</v>
@@ -13764,16 +13656,14 @@
       </c>
       <c r="E291" t="inlineStr"/>
       <c r="F291" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G291" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H291" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H291" s="3" t="n"/>
       <c r="I291" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J291" s="2" t="n">
         <v>23.99</v>
@@ -13904,16 +13794,14 @@
       </c>
       <c r="E294" t="inlineStr"/>
       <c r="F294" s="2" t="n">
-        <v>19.99</v>
+        <v>22.99</v>
       </c>
       <c r="G294" s="2" t="n">
         <v>22.99</v>
       </c>
-      <c r="H294" s="3" t="n">
-        <v>15</v>
-      </c>
+      <c r="H294" s="3" t="n"/>
       <c r="I294" s="2" t="n">
-        <v>21.99</v>
+        <v>25.49</v>
       </c>
       <c r="J294" s="2" t="n">
         <v>25.49</v>
@@ -14084,16 +13972,14 @@
       </c>
       <c r="E298" t="inlineStr"/>
       <c r="F298" s="2" t="n">
-        <v>10.99</v>
+        <v>11.99</v>
       </c>
       <c r="G298" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H298" s="3" t="n">
-        <v>9.1</v>
-      </c>
+      <c r="H298" s="3" t="n"/>
       <c r="I298" s="2" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="J298" s="2" t="n">
         <v>12.99</v>
@@ -14132,16 +14018,14 @@
       </c>
       <c r="E299" t="inlineStr"/>
       <c r="F299" s="2" t="n">
-        <v>28.99</v>
+        <v>23.99</v>
       </c>
       <c r="G299" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H299" s="3" t="n">
-        <v>-17.2</v>
-      </c>
+      <c r="H299" s="3" t="n"/>
       <c r="I299" s="2" t="n">
-        <v>29.99</v>
+        <v>24.99</v>
       </c>
       <c r="J299" s="2" t="n">
         <v>24.99</v>
@@ -14180,16 +14064,14 @@
       </c>
       <c r="E300" t="inlineStr"/>
       <c r="F300" s="2" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="G300" s="2" t="n">
         <v>12.99</v>
       </c>
-      <c r="H300" s="3" t="n">
-        <v>8.300000000000001</v>
-      </c>
+      <c r="H300" s="3" t="n"/>
       <c r="I300" s="2" t="n">
-        <v>12.99</v>
+        <v>13.99</v>
       </c>
       <c r="J300" s="2" t="n">
         <v>13.99</v>
@@ -14272,16 +14154,14 @@
       </c>
       <c r="E302" t="inlineStr"/>
       <c r="F302" s="2" t="n">
-        <v>8.99</v>
+        <v>11.99</v>
       </c>
       <c r="G302" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H302" s="3" t="n">
-        <v>33.4</v>
-      </c>
+      <c r="H302" s="3" t="n"/>
       <c r="I302" s="2" t="n">
-        <v>9.99</v>
+        <v>13.49</v>
       </c>
       <c r="J302" s="2" t="n">
         <v>13.49</v>
@@ -14364,16 +14244,14 @@
       </c>
       <c r="E304" t="inlineStr"/>
       <c r="F304" s="2" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="G304" s="2" t="n">
         <v>12.99</v>
       </c>
-      <c r="H304" s="3" t="n">
-        <v>8.300000000000001</v>
-      </c>
+      <c r="H304" s="3" t="n"/>
       <c r="I304" s="2" t="n">
-        <v>12.99</v>
+        <v>13.99</v>
       </c>
       <c r="J304" s="2" t="n">
         <v>13.99</v>
@@ -14412,16 +14290,14 @@
       </c>
       <c r="E305" t="inlineStr"/>
       <c r="F305" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="G305" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H305" s="3" t="n">
-        <v>9.1</v>
-      </c>
+      <c r="H305" s="3" t="n"/>
       <c r="I305" s="2" t="n">
-        <v>23.99</v>
+        <v>25.99</v>
       </c>
       <c r="J305" s="2" t="n">
         <v>25.99</v>
@@ -15331,7 +15207,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -15383,16 +15259,14 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>24.99</v>
+        <v>29.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>29.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>20</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
-        <v>27.49</v>
+        <v>32.99</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>32.99</v>
@@ -15431,16 +15305,14 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>18.49</v>
@@ -15479,16 +15351,14 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>18.49</v>
@@ -15527,16 +15397,14 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>18.49</v>
@@ -15575,16 +15443,14 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>14.99</v>
+        <v>16.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>16.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>13.3</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
-        <v>16.49</v>
+        <v>18.49</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>18.49</v>
@@ -15623,16 +15489,14 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>19.99</v>
+        <v>22.99</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>22.99</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>15</v>
-      </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
-        <v>21.99</v>
+        <v>25.49</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>25.49</v>
@@ -15710,7 +15574,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -15991,7 +15855,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -16266,7 +16130,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -16318,16 +16182,14 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>19.99</v>
+        <v>22.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>22.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>15</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
-        <v>21.99</v>
+        <v>25.49</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>25.49</v>
@@ -16405,7 +16267,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -16503,16 +16365,14 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>19.49</v>
@@ -16793,16 +16653,14 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H9" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>19.49</v>
@@ -17083,16 +16941,14 @@
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H15" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>21.99</v>
@@ -17223,16 +17079,14 @@
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H18" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>19.49</v>
@@ -17607,16 +17461,14 @@
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H26" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H26" s="3" t="n"/>
       <c r="I26" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>21.99</v>
@@ -17655,16 +17507,14 @@
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>31.99</v>
+        <v>34.99</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H27" s="3" t="n">
-        <v>9.4</v>
-      </c>
+      <c r="H27" s="3" t="n"/>
       <c r="I27" s="2" t="n">
-        <v>34.99</v>
+        <v>38.49</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>38.49</v>
@@ -17979,16 +17829,14 @@
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="n">
-        <v>31.99</v>
+        <v>34.99</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H34" s="3" t="n">
-        <v>9.4</v>
-      </c>
+      <c r="H34" s="3" t="n"/>
       <c r="I34" s="2" t="n">
-        <v>34.99</v>
+        <v>38.49</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>38.49</v>
@@ -18775,16 +18623,14 @@
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H51" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H51" s="3" t="n"/>
       <c r="I51" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>23.99</v>
@@ -18869,16 +18715,14 @@
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H53" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H53" s="3" t="n"/>
       <c r="I53" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>19.49</v>
@@ -18963,16 +18807,14 @@
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H55" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H55" s="3" t="n"/>
       <c r="I55" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>19.49</v>
@@ -19011,16 +18853,14 @@
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" s="2" t="n">
-        <v>24.99</v>
+        <v>27.99</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H56" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="H56" s="3" t="n"/>
       <c r="I56" s="2" t="n">
-        <v>27.49</v>
+        <v>30.99</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>30.99</v>
@@ -19385,16 +19225,14 @@
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H64" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H64" s="3" t="n"/>
       <c r="I64" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>19.49</v>
@@ -19433,16 +19271,14 @@
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" s="2" t="n">
-        <v>21.99</v>
+        <v>27.99</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H65" s="3" t="n">
-        <v>27.3</v>
-      </c>
+      <c r="H65" s="3" t="n"/>
       <c r="I65" s="2" t="n">
-        <v>23.99</v>
+        <v>30.49</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>30.49</v>
@@ -19619,16 +19455,14 @@
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H69" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H69" s="3" t="n"/>
       <c r="I69" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>19.49</v>
@@ -19713,16 +19547,14 @@
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H71" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H71" s="3" t="n"/>
       <c r="I71" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>19.49</v>
@@ -19853,16 +19685,14 @@
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G74" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H74" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H74" s="3" t="n"/>
       <c r="I74" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>21.99</v>
@@ -19947,16 +19777,14 @@
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H76" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H76" s="3" t="n"/>
       <c r="I76" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>19.49</v>
@@ -20575,16 +20403,14 @@
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G89" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H89" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H89" s="3" t="n"/>
       <c r="I89" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>23.99</v>
@@ -20669,16 +20495,14 @@
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G91" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H91" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H91" s="3" t="n"/>
       <c r="I91" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>19.49</v>
@@ -20717,16 +20541,14 @@
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" s="2" t="n">
-        <v>24.99</v>
+        <v>27.99</v>
       </c>
       <c r="G92" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H92" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="H92" s="3" t="n"/>
       <c r="I92" s="2" t="n">
-        <v>27.49</v>
+        <v>30.99</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>30.99</v>
@@ -21559,16 +21381,14 @@
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G110" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H110" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H110" s="3" t="n"/>
       <c r="I110" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>21.99</v>
@@ -21699,16 +21519,14 @@
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G113" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H113" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H113" s="3" t="n"/>
       <c r="I113" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>19.49</v>
@@ -21747,16 +21565,14 @@
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" s="2" t="n">
-        <v>24.99</v>
+        <v>27.99</v>
       </c>
       <c r="G114" s="2" t="n">
         <v>27.99</v>
       </c>
-      <c r="H114" s="3" t="n">
-        <v>12</v>
-      </c>
+      <c r="H114" s="3" t="n"/>
       <c r="I114" s="2" t="n">
-        <v>27.49</v>
+        <v>30.99</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>30.99</v>
@@ -21880,7 +21696,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -22070,16 +21886,14 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>19.49</v>
@@ -22538,16 +22352,14 @@
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H15" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>21.99</v>
@@ -22586,16 +22398,14 @@
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>29.99</v>
+        <v>32.99</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>32.99</v>
       </c>
-      <c r="H16" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
-        <v>32.99</v>
+        <v>36.49</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>36.49</v>
@@ -22680,16 +22490,14 @@
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H18" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>21.99</v>
@@ -22820,16 +22628,14 @@
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>29.99</v>
+        <v>32.99</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>32.99</v>
       </c>
-      <c r="H21" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H21" s="3" t="n"/>
       <c r="I21" s="2" t="n">
-        <v>32.99</v>
+        <v>36.49</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>36.49</v>
@@ -23236,16 +23042,14 @@
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H30" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H30" s="3" t="n"/>
       <c r="I30" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>21.99</v>
@@ -23376,16 +23180,14 @@
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H33" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H33" s="3" t="n"/>
       <c r="I33" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>19.49</v>
@@ -23470,16 +23272,14 @@
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H35" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H35" s="3" t="n"/>
       <c r="I35" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>19.49</v>
@@ -23518,16 +23318,14 @@
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H36" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H36" s="3" t="n"/>
       <c r="I36" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>25.99</v>
@@ -23612,16 +23410,14 @@
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H38" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H38" s="3" t="n"/>
       <c r="I38" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>19.49</v>
@@ -23752,16 +23548,14 @@
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H41" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H41" s="3" t="n"/>
       <c r="I41" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>25.99</v>
@@ -23800,16 +23594,14 @@
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H42" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H42" s="3" t="n"/>
       <c r="I42" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>21.99</v>
@@ -24032,16 +23824,14 @@
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H47" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H47" s="3" t="n"/>
       <c r="I47" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>21.99</v>
@@ -24552,16 +24342,14 @@
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H58" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H58" s="3" t="n"/>
       <c r="I58" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>23.99</v>
@@ -24600,16 +24388,14 @@
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H59" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H59" s="3" t="n"/>
       <c r="I59" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>19.49</v>
@@ -24648,16 +24434,14 @@
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H60" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H60" s="3" t="n"/>
       <c r="I60" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>25.99</v>
@@ -25248,16 +25032,14 @@
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>19.99</v>
       </c>
-      <c r="H73" s="3" t="n">
-        <v>5.3</v>
-      </c>
+      <c r="H73" s="3" t="n"/>
       <c r="I73" s="2" t="n">
-        <v>20.99</v>
+        <v>21.99</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>21.99</v>
@@ -25342,16 +25124,14 @@
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H75" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H75" s="3" t="n"/>
       <c r="I75" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>19.49</v>
@@ -25390,16 +25170,14 @@
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" s="2" t="n">
-        <v>21.49</v>
+        <v>23.99</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H76" s="3" t="n">
-        <v>11.6</v>
-      </c>
+      <c r="H76" s="3" t="n"/>
       <c r="I76" s="2" t="n">
-        <v>23.49</v>
+        <v>25.99</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>25.99</v>
@@ -25477,7 +25255,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -26301,16 +26079,14 @@
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>34.99</v>
+        <v>37.99</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>37.99</v>
       </c>
-      <c r="H20" s="3" t="n">
-        <v>8.6</v>
-      </c>
+      <c r="H20" s="3" t="n"/>
       <c r="I20" s="2" t="n">
-        <v>38.49</v>
+        <v>41.99</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>41.99</v>
@@ -27584,7 +27360,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -27768,16 +27544,14 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>10.99</v>
+        <v>11.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>9.1</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>12.99</v>
@@ -27816,16 +27590,14 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>28.99</v>
+        <v>23.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>-17.2</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
-        <v>29.99</v>
+        <v>24.99</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>24.99</v>
@@ -27864,16 +27636,14 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>12.99</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>8.300000000000001</v>
-      </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
-        <v>12.99</v>
+        <v>13.99</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>13.99</v>
@@ -27956,16 +27726,14 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>8.99</v>
+        <v>11.99</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H9" s="3" t="n">
-        <v>33.4</v>
-      </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>9.99</v>
+        <v>13.49</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>13.49</v>
@@ -28048,16 +27816,14 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>12.99</v>
       </c>
-      <c r="H11" s="3" t="n">
-        <v>8.300000000000001</v>
-      </c>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>12.99</v>
+        <v>13.99</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>13.99</v>
@@ -28096,16 +27862,14 @@
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>23.99</v>
       </c>
-      <c r="H12" s="3" t="n">
-        <v>9.1</v>
-      </c>
+      <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>23.99</v>
+        <v>25.99</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>25.99</v>
@@ -28663,7 +28427,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -29636,7 +29400,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -29950,16 +29714,14 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>24.99</v>
+        <v>29.99</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>29.99</v>
       </c>
-      <c r="H8" s="3" t="n">
-        <v>20</v>
-      </c>
+      <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
-        <v>27.49</v>
+        <v>32.99</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>32.99</v>
@@ -30291,7 +30053,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -30734,7 +30496,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price 2026-09-15</t>
+          <t>Price 2026-09-18</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -30786,16 +30548,14 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>22.99</v>
+        <v>24.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>24.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>8.699999999999999</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
-        <v>25.49</v>
+        <v>27.49</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>27.49</v>
@@ -30834,16 +30594,14 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>23.99</v>
@@ -30882,16 +30640,14 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>23.99</v>
@@ -30930,16 +30686,14 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>23.99</v>
@@ -30978,16 +30732,14 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>19.99</v>
+        <v>21.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>21.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>10</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
-        <v>21.99</v>
+        <v>23.99</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>23.99</v>

</xml_diff>

<commit_message>
Price list: derived half applied; restore the excluded-rows marker
The 79-row derived increase is live, so the page now shows 0 pending changes.
Also fixes a reporting defect the staging run introduced: my staged plan dropped
the source plan's excluded array, and build_price_list_report keys
'Held - excluded by Justin' off it. Without it the two Worldwide Botanicals rows
Justin excluded by name on 2026-09-14 fell through to the derived-ladder fallback
and were published as a proposed $11.99 increase on another brand's product.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/shopify-price-list.xlsx
+++ b/shopify-price-list.xlsx
@@ -550,14 +550,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>31.5</v>
+        <v>33.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>33.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>7.9</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" t="inlineStr">
@@ -700,14 +698,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>50</v>
+        <v>53.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
         <v>0</v>
       </c>
@@ -1626,16 +1622,14 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H28" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H28" s="3" t="n"/>
       <c r="I28" s="2" t="n">
-        <v>57.96</v>
+        <v>62.49</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>62.49</v>
@@ -1670,16 +1664,14 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" s="2" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>43.99</v>
       </c>
-      <c r="H29" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H29" s="3" t="n"/>
       <c r="I29" s="2" t="n">
-        <v>52.97</v>
+        <v>56.99</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>56.99</v>
@@ -1714,16 +1706,14 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H30" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H30" s="3" t="n"/>
       <c r="I30" s="2" t="n">
-        <v>52.97</v>
+        <v>56.49</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>56.49</v>
@@ -1758,14 +1748,12 @@
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
       <c r="F31" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H31" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H31" s="3" t="n"/>
       <c r="I31" s="2" t="n">
         <v>0</v>
       </c>
@@ -1802,14 +1790,12 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H32" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H32" s="3" t="n"/>
       <c r="I32" s="2" t="n">
         <v>0</v>
       </c>
@@ -1846,14 +1832,12 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H33" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H33" s="3" t="n"/>
       <c r="I33" s="2" t="n">
         <v>0</v>
       </c>
@@ -1890,14 +1874,12 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H34" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H34" s="3" t="n"/>
       <c r="I34" s="2" t="n">
         <v>0</v>
       </c>
@@ -1934,14 +1916,12 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H35" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H35" s="3" t="n"/>
       <c r="I35" s="2" t="n">
         <v>0</v>
       </c>
@@ -1978,14 +1958,12 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H36" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H36" s="3" t="n"/>
       <c r="I36" s="2" t="n">
         <v>0</v>
       </c>
@@ -2022,16 +2000,14 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H37" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H37" s="3" t="n"/>
       <c r="I37" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>80.98999999999999</v>
@@ -2062,16 +2038,14 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H38" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H38" s="3" t="n"/>
       <c r="I38" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>80.48999999999999</v>
@@ -2102,16 +2076,14 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H39" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H39" s="3" t="n"/>
       <c r="I39" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>80.98999999999999</v>
@@ -2142,16 +2114,14 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H40" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H40" s="3" t="n"/>
       <c r="I40" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>80.48999999999999</v>
@@ -2186,14 +2156,12 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" s="2" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>43.99</v>
       </c>
-      <c r="H41" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H41" s="3" t="n"/>
       <c r="I41" s="2" t="n"/>
       <c r="J41" s="2" t="n"/>
       <c r="K41" t="inlineStr">
@@ -2226,14 +2194,12 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H42" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H42" s="3" t="n"/>
       <c r="I42" s="2" t="n"/>
       <c r="J42" s="2" t="n"/>
       <c r="K42" t="inlineStr">
@@ -2266,14 +2232,12 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H43" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H43" s="3" t="n"/>
       <c r="I43" s="2" t="n">
         <v>0</v>
       </c>
@@ -2310,14 +2274,12 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
       <c r="F44" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H44" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H44" s="3" t="n"/>
       <c r="I44" s="2" t="n">
         <v>0</v>
       </c>
@@ -2354,14 +2316,12 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H45" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H45" s="3" t="n"/>
       <c r="I45" s="2" t="n">
         <v>0</v>
       </c>
@@ -2444,14 +2404,12 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H47" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H47" s="3" t="n"/>
       <c r="I47" s="2" t="n">
         <v>0</v>
       </c>
@@ -2488,14 +2446,12 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
       <c r="F48" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H48" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H48" s="3" t="n"/>
       <c r="I48" s="2" t="n">
         <v>0</v>
       </c>
@@ -2532,14 +2488,12 @@
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H49" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H49" s="3" t="n"/>
       <c r="I49" s="2" t="n">
         <v>0</v>
       </c>
@@ -2576,14 +2530,12 @@
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
       <c r="F50" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H50" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H50" s="3" t="n"/>
       <c r="I50" s="2" t="n">
         <v>0</v>
       </c>
@@ -2616,16 +2568,14 @@
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H51" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H51" s="3" t="n"/>
       <c r="I51" s="2" t="n">
-        <v>54.99</v>
+        <v>59.49</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>59.49</v>
@@ -2660,16 +2610,14 @@
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
       <c r="F52" s="2" t="n">
-        <v>69.98999999999999</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>74.98999999999999</v>
       </c>
-      <c r="H52" s="3" t="n">
-        <v>7.1</v>
-      </c>
+      <c r="H52" s="3" t="n"/>
       <c r="I52" s="2" t="n">
-        <v>94.95999999999999</v>
+        <v>101.99</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>101.99</v>
@@ -2704,16 +2652,14 @@
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
       <c r="F53" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H53" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H53" s="3" t="n"/>
       <c r="I53" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>80.48999999999999</v>
@@ -2748,16 +2694,14 @@
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H54" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H54" s="3" t="n"/>
       <c r="I54" s="2" t="n">
-        <v>54.99</v>
+        <v>59.49</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>59.49</v>
@@ -2792,16 +2736,14 @@
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H55" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H55" s="3" t="n"/>
       <c r="I55" s="2" t="n">
-        <v>54.99</v>
+        <v>59.49</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>59.49</v>
@@ -2920,16 +2862,14 @@
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr"/>
       <c r="F58" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H58" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H58" s="3" t="n"/>
       <c r="I58" s="2" t="n">
-        <v>49.49</v>
+        <v>52.99</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>52.99</v>
@@ -2960,16 +2900,14 @@
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr"/>
       <c r="F59" s="2" t="n">
-        <v>55.99</v>
+        <v>56.99</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>56.99</v>
       </c>
-      <c r="H59" s="3" t="n">
-        <v>1.8</v>
-      </c>
+      <c r="H59" s="3" t="n"/>
       <c r="I59" s="2" t="n">
-        <v>71.95</v>
+        <v>73.48999999999999</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>73.48999999999999</v>
@@ -3004,16 +2942,14 @@
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
       <c r="F60" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H60" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H60" s="3" t="n"/>
       <c r="I60" s="2" t="n">
-        <v>50.97</v>
+        <v>54.99</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>54.99</v>
@@ -3048,14 +2984,12 @@
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
       <c r="F61" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H61" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H61" s="3" t="n"/>
       <c r="I61" s="2" t="n">
         <v>0</v>
       </c>
@@ -3092,16 +3026,14 @@
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
       <c r="F62" s="2" t="n">
-        <v>59.99</v>
+        <v>63.99</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>63.99</v>
       </c>
-      <c r="H62" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H62" s="3" t="n"/>
       <c r="I62" s="2" t="n">
-        <v>80.95999999999999</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>86.48999999999999</v>
@@ -3136,16 +3068,14 @@
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
       <c r="F63" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H63" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H63" s="3" t="n"/>
       <c r="I63" s="2" t="n">
-        <v>56.96</v>
+        <v>60.99</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>60.99</v>
@@ -3180,14 +3110,12 @@
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
       <c r="F64" s="2" t="n">
-        <v>52.99</v>
+        <v>56.99</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>56.99</v>
       </c>
-      <c r="H64" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H64" s="3" t="n"/>
       <c r="I64" s="2" t="n">
         <v>0</v>
       </c>
@@ -3224,16 +3152,14 @@
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
       <c r="F65" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H65" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H65" s="3" t="n"/>
       <c r="I65" s="2" t="n">
-        <v>64.95999999999999</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>69.98999999999999</v>
@@ -3264,16 +3190,14 @@
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
       <c r="F66" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H66" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H66" s="3" t="n"/>
       <c r="I66" s="2" t="n">
-        <v>64.95999999999999</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>69.98999999999999</v>
@@ -3308,16 +3232,14 @@
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
       <c r="F67" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H67" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H67" s="3" t="n"/>
       <c r="I67" s="2" t="n">
-        <v>61.26</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>65.98999999999999</v>
@@ -3348,16 +3270,14 @@
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
       <c r="F68" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H68" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H68" s="3" t="n"/>
       <c r="I68" s="2" t="n">
-        <v>51.27</v>
+        <v>55.49</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>55.49</v>
@@ -3392,16 +3312,14 @@
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
       <c r="F69" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H69" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H69" s="3" t="n"/>
       <c r="I69" s="2" t="n">
-        <v>62.96</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>67.98999999999999</v>
@@ -3432,16 +3350,14 @@
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr"/>
       <c r="F70" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G70" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H70" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H70" s="3" t="n"/>
       <c r="I70" s="2" t="n">
-        <v>62.96</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>67.98999999999999</v>
@@ -3472,16 +3388,14 @@
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
       <c r="F71" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H71" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H71" s="3" t="n"/>
       <c r="I71" s="2" t="n">
-        <v>65.95</v>
+        <v>70.98999999999999</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>70.98999999999999</v>
@@ -3512,16 +3426,14 @@
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
       <c r="F72" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H72" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H72" s="3" t="n"/>
       <c r="I72" s="2" t="n">
-        <v>55.97</v>
+        <v>60.49</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>60.49</v>
@@ -3556,16 +3468,14 @@
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
       <c r="F73" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H73" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H73" s="3" t="n"/>
       <c r="I73" s="2" t="n">
-        <v>63.96</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>68.98999999999999</v>
@@ -3596,16 +3506,14 @@
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
       <c r="F74" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G74" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H74" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H74" s="3" t="n"/>
       <c r="I74" s="2" t="n">
-        <v>53.97</v>
+        <v>58.49</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>58.49</v>
@@ -3644,16 +3552,14 @@
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" s="2" t="n">
-        <v>12.99</v>
+        <v>13.99</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>13.99</v>
       </c>
-      <c r="H75" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H75" s="3" t="n"/>
       <c r="I75" s="2" t="n">
-        <v>14.49</v>
+        <v>15.49</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>15.49</v>
@@ -3738,17 +3644,13 @@
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" s="2" t="n">
-        <v>9.99</v>
+        <v>10.99</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>10.99</v>
       </c>
-      <c r="H77" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="I77" s="2" t="n">
-        <v>9.99</v>
-      </c>
+      <c r="H77" s="3" t="n"/>
+      <c r="I77" s="2" t="n"/>
       <c r="J77" s="2" t="n"/>
       <c r="K77" t="inlineStr">
         <is>
@@ -3780,16 +3682,14 @@
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
       <c r="F78" s="2" t="n">
-        <v>17.99</v>
+        <v>18.99</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>18.99</v>
       </c>
-      <c r="H78" s="3" t="n">
-        <v>5.6</v>
-      </c>
+      <c r="H78" s="3" t="n"/>
       <c r="I78" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>19.99</v>
@@ -3866,14 +3766,12 @@
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
       <c r="F80" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G80" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H80" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H80" s="3" t="n"/>
       <c r="I80" s="2" t="n">
         <v>0</v>
       </c>
@@ -3910,14 +3808,12 @@
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
       <c r="F81" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G81" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H81" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H81" s="3" t="n"/>
       <c r="I81" s="2" t="n">
         <v>0</v>
       </c>
@@ -3954,14 +3850,12 @@
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
       <c r="F82" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G82" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H82" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H82" s="3" t="n"/>
       <c r="I82" s="2" t="n">
         <v>0</v>
       </c>
@@ -3998,14 +3892,12 @@
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
       <c r="F83" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G83" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H83" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H83" s="3" t="n"/>
       <c r="I83" s="2" t="n">
         <v>0</v>
       </c>
@@ -4042,16 +3934,14 @@
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
       <c r="F84" s="2" t="n">
-        <v>33.99</v>
+        <v>36.99</v>
       </c>
       <c r="G84" s="2" t="n">
         <v>36.99</v>
       </c>
-      <c r="H84" s="3" t="n">
-        <v>8.800000000000001</v>
-      </c>
+      <c r="H84" s="3" t="n"/>
       <c r="I84" s="2" t="n">
-        <v>35.99</v>
+        <v>38.99</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>38.99</v>
@@ -4132,16 +4022,14 @@
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr"/>
       <c r="F86" s="2" t="n">
-        <v>119.99</v>
+        <v>128.99</v>
       </c>
       <c r="G86" s="2" t="n">
         <v>128.99</v>
       </c>
-      <c r="H86" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H86" s="3" t="n"/>
       <c r="I86" s="2" t="n">
-        <v>131.99</v>
+        <v>141.99</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>141.99</v>
@@ -5292,16 +5180,14 @@
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G111" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H111" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H111" s="3" t="n"/>
       <c r="I111" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>19.49</v>
@@ -10100,16 +9986,14 @@
       </c>
       <c r="E214" t="inlineStr"/>
       <c r="F214" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G214" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H214" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H214" s="3" t="n"/>
       <c r="I214" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J214" s="2" t="n">
         <v>19.49</v>
@@ -12552,16 +12436,14 @@
       <c r="D267" t="inlineStr"/>
       <c r="E267" t="inlineStr"/>
       <c r="F267" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G267" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H267" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H267" s="3" t="n"/>
       <c r="I267" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="J267" s="2" t="n">
         <v>19.99</v>
@@ -12780,16 +12662,14 @@
       <c r="D272" t="inlineStr"/>
       <c r="E272" t="inlineStr"/>
       <c r="F272" s="2" t="n">
-        <v>14.49</v>
+        <v>15.99</v>
       </c>
       <c r="G272" s="2" t="n">
         <v>15.99</v>
       </c>
-      <c r="H272" s="3" t="n">
-        <v>10.4</v>
-      </c>
+      <c r="H272" s="3" t="n"/>
       <c r="I272" s="2" t="n">
-        <v>14.99</v>
+        <v>16.49</v>
       </c>
       <c r="J272" s="2" t="n">
         <v>16.49</v>
@@ -13836,16 +13716,14 @@
       <c r="D295" t="inlineStr"/>
       <c r="E295" t="inlineStr"/>
       <c r="F295" s="2" t="n">
-        <v>31.99</v>
+        <v>33.99</v>
       </c>
       <c r="G295" s="2" t="n">
         <v>33.99</v>
       </c>
-      <c r="H295" s="3" t="n">
-        <v>6.3</v>
-      </c>
+      <c r="H295" s="3" t="n"/>
       <c r="I295" s="2" t="n">
-        <v>34.99</v>
+        <v>36.99</v>
       </c>
       <c r="J295" s="2" t="n">
         <v>36.99</v>
@@ -13880,16 +13758,14 @@
       <c r="D296" t="inlineStr"/>
       <c r="E296" t="inlineStr"/>
       <c r="F296" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G296" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H296" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H296" s="3" t="n"/>
       <c r="I296" s="2" t="n">
-        <v>21.99</v>
+        <v>22.99</v>
       </c>
       <c r="J296" s="2" t="n">
         <v>22.99</v>
@@ -13924,16 +13800,14 @@
       <c r="D297" t="inlineStr"/>
       <c r="E297" t="inlineStr"/>
       <c r="F297" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G297" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H297" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H297" s="3" t="n"/>
       <c r="I297" s="2" t="n">
-        <v>21.99</v>
+        <v>22.99</v>
       </c>
       <c r="J297" s="2" t="n">
         <v>22.99</v>
@@ -14106,14 +13980,12 @@
       <c r="D301" t="inlineStr"/>
       <c r="E301" t="inlineStr"/>
       <c r="F301" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G301" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H301" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H301" s="3" t="n"/>
       <c r="I301" s="2" t="n">
         <v>0</v>
       </c>
@@ -14196,16 +14068,14 @@
       <c r="D303" t="inlineStr"/>
       <c r="E303" t="inlineStr"/>
       <c r="F303" s="2" t="n">
-        <v>9.56</v>
+        <v>9.99</v>
       </c>
       <c r="G303" s="2" t="n">
         <v>9.99</v>
       </c>
-      <c r="H303" s="3" t="n">
-        <v>4.5</v>
-      </c>
+      <c r="H303" s="3" t="n"/>
       <c r="I303" s="2" t="n">
-        <v>9.99</v>
+        <v>10.49</v>
       </c>
       <c r="J303" s="2" t="n">
         <v>10.49</v>
@@ -14332,16 +14202,14 @@
       <c r="D306" t="inlineStr"/>
       <c r="E306" t="inlineStr"/>
       <c r="F306" s="2" t="n">
-        <v>14.99</v>
+        <v>15.99</v>
       </c>
       <c r="G306" s="2" t="n">
         <v>15.99</v>
       </c>
-      <c r="H306" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H306" s="3" t="n"/>
       <c r="I306" s="2" t="n">
-        <v>20.99</v>
+        <v>22.49</v>
       </c>
       <c r="J306" s="2" t="n">
         <v>22.49</v>
@@ -14464,14 +14332,12 @@
       <c r="D309" t="inlineStr"/>
       <c r="E309" t="inlineStr"/>
       <c r="F309" s="2" t="n">
-        <v>10.95</v>
+        <v>11.99</v>
       </c>
       <c r="G309" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H309" s="3" t="n">
-        <v>9.5</v>
-      </c>
+      <c r="H309" s="3" t="n"/>
       <c r="I309" s="2" t="n">
         <v>0</v>
       </c>
@@ -14508,14 +14374,12 @@
       <c r="D310" t="inlineStr"/>
       <c r="E310" t="inlineStr"/>
       <c r="F310" s="2" t="n">
-        <v>10.95</v>
+        <v>11.99</v>
       </c>
       <c r="G310" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H310" s="3" t="n">
-        <v>9.5</v>
-      </c>
+      <c r="H310" s="3" t="n"/>
       <c r="I310" s="2" t="n">
         <v>0</v>
       </c>
@@ -14552,14 +14416,12 @@
       <c r="D311" t="inlineStr"/>
       <c r="E311" t="inlineStr"/>
       <c r="F311" s="2" t="n">
-        <v>28.99</v>
+        <v>30.99</v>
       </c>
       <c r="G311" s="2" t="n">
         <v>30.99</v>
       </c>
-      <c r="H311" s="3" t="n">
-        <v>6.9</v>
-      </c>
+      <c r="H311" s="3" t="n"/>
       <c r="I311" s="2" t="n">
         <v>0</v>
       </c>
@@ -14596,14 +14458,12 @@
       <c r="D312" t="inlineStr"/>
       <c r="E312" t="inlineStr"/>
       <c r="F312" s="2" t="n">
-        <v>9.56</v>
+        <v>9.99</v>
       </c>
       <c r="G312" s="2" t="n">
         <v>9.99</v>
       </c>
-      <c r="H312" s="3" t="n">
-        <v>4.5</v>
-      </c>
+      <c r="H312" s="3" t="n"/>
       <c r="I312" s="2" t="n">
         <v>0</v>
       </c>
@@ -14640,14 +14500,12 @@
       <c r="D313" t="inlineStr"/>
       <c r="E313" t="inlineStr"/>
       <c r="F313" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G313" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H313" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H313" s="3" t="n"/>
       <c r="I313" s="2" t="n">
         <v>0</v>
       </c>
@@ -14684,16 +14542,14 @@
       <c r="D314" t="inlineStr"/>
       <c r="E314" t="inlineStr"/>
       <c r="F314" s="2" t="n">
-        <v>29.99</v>
+        <v>31.99</v>
       </c>
       <c r="G314" s="2" t="n">
         <v>31.99</v>
       </c>
-      <c r="H314" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H314" s="3" t="n"/>
       <c r="I314" s="2" t="n">
-        <v>32.99</v>
+        <v>34.99</v>
       </c>
       <c r="J314" s="2" t="n">
         <v>34.99</v>
@@ -14812,16 +14668,14 @@
       <c r="D317" t="inlineStr"/>
       <c r="E317" t="inlineStr"/>
       <c r="F317" s="2" t="n">
-        <v>55.99</v>
+        <v>59.99</v>
       </c>
       <c r="G317" s="2" t="n">
         <v>59.99</v>
       </c>
-      <c r="H317" s="3" t="n">
-        <v>7.1</v>
-      </c>
+      <c r="H317" s="3" t="n"/>
       <c r="I317" s="2" t="n">
-        <v>58.99</v>
+        <v>62.99</v>
       </c>
       <c r="J317" s="2" t="n">
         <v>62.99</v>
@@ -14856,16 +14710,14 @@
       <c r="D318" t="inlineStr"/>
       <c r="E318" t="inlineStr"/>
       <c r="F318" s="2" t="n">
-        <v>33.99</v>
+        <v>34.99</v>
       </c>
       <c r="G318" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H318" s="3" t="n">
-        <v>2.9</v>
-      </c>
+      <c r="H318" s="3" t="n"/>
       <c r="I318" s="2" t="n">
-        <v>37.49</v>
+        <v>38.49</v>
       </c>
       <c r="J318" s="2" t="n">
         <v>38.49</v>
@@ -14900,16 +14752,14 @@
       <c r="D319" t="inlineStr"/>
       <c r="E319" t="inlineStr"/>
       <c r="F319" s="2" t="n">
-        <v>63.99</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="G319" s="2" t="n">
         <v>68.98999999999999</v>
       </c>
-      <c r="H319" s="3" t="n">
-        <v>7.8</v>
-      </c>
+      <c r="H319" s="3" t="n"/>
       <c r="I319" s="2" t="n">
-        <v>70.48999999999999</v>
+        <v>75.98999999999999</v>
       </c>
       <c r="J319" s="2" t="n">
         <v>75.98999999999999</v>
@@ -14944,16 +14794,14 @@
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr"/>
       <c r="F320" s="2" t="n">
-        <v>32.99</v>
+        <v>34.99</v>
       </c>
       <c r="G320" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H320" s="3" t="n">
-        <v>6.1</v>
-      </c>
+      <c r="H320" s="3" t="n"/>
       <c r="I320" s="2" t="n">
-        <v>34.99</v>
+        <v>36.99</v>
       </c>
       <c r="J320" s="2" t="n">
         <v>36.99</v>
@@ -14988,16 +14836,14 @@
       <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr"/>
       <c r="F321" s="2" t="n">
-        <v>56.99</v>
+        <v>60.99</v>
       </c>
       <c r="G321" s="2" t="n">
         <v>60.99</v>
       </c>
-      <c r="H321" s="3" t="n">
-        <v>7</v>
-      </c>
+      <c r="H321" s="3" t="n"/>
       <c r="I321" s="2" t="n">
-        <v>62.49</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="J321" s="2" t="n">
         <v>66.98999999999999</v>
@@ -15032,16 +14878,14 @@
       <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr"/>
       <c r="F322" s="2" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="G322" s="2" t="n">
         <v>43.99</v>
       </c>
-      <c r="H322" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H322" s="3" t="n"/>
       <c r="I322" s="2" t="n">
-        <v>42.99</v>
+        <v>45.99</v>
       </c>
       <c r="J322" s="2" t="n">
         <v>45.99</v>
@@ -15076,16 +14920,14 @@
       <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr"/>
       <c r="F323" s="2" t="n">
-        <v>41.99</v>
+        <v>44.99</v>
       </c>
       <c r="G323" s="2" t="n">
         <v>44.99</v>
       </c>
-      <c r="H323" s="3" t="n">
-        <v>7.1</v>
-      </c>
+      <c r="H323" s="3" t="n"/>
       <c r="I323" s="2" t="n">
-        <v>43.99</v>
+        <v>46.99</v>
       </c>
       <c r="J323" s="2" t="n">
         <v>46.99</v>
@@ -15120,16 +14962,14 @@
       <c r="D324" t="inlineStr"/>
       <c r="E324" t="inlineStr"/>
       <c r="F324" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G324" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H324" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H324" s="3" t="n"/>
       <c r="I324" s="2" t="n">
-        <v>73.95999999999999</v>
+        <v>79.48999999999999</v>
       </c>
       <c r="J324" s="2" t="n">
         <v>79.48999999999999</v>
@@ -15618,14 +15458,12 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>31.5</v>
+        <v>33.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>33.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>7.9</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" t="inlineStr">
@@ -15768,14 +15606,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>50</v>
+        <v>53.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
         <v>0</v>
       </c>
@@ -15907,16 +15743,14 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>12.99</v>
+        <v>13.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>13.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
-        <v>14.49</v>
+        <v>15.49</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>15.49</v>
@@ -16001,17 +15835,13 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>9.99</v>
+        <v>10.99</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>10.99</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>9.99</v>
-      </c>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="n"/>
       <c r="K4" t="inlineStr">
         <is>
@@ -16043,16 +15873,14 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>17.99</v>
+        <v>18.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>18.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>5.6</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>19.99</v>
@@ -17221,16 +17049,14 @@
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H21" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H21" s="3" t="n"/>
       <c r="I21" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>19.49</v>
@@ -22120,16 +21946,14 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H10" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
-        <v>18.49</v>
+        <v>19.49</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>19.49</v>
@@ -24572,16 +24396,14 @@
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
       <c r="F63" s="2" t="n">
-        <v>16.99</v>
+        <v>17.99</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>17.99</v>
       </c>
-      <c r="H63" s="3" t="n">
-        <v>5.9</v>
-      </c>
+      <c r="H63" s="3" t="n"/>
       <c r="I63" s="2" t="n">
-        <v>18.99</v>
+        <v>19.99</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>19.99</v>
@@ -24800,16 +24622,14 @@
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
       <c r="F68" s="2" t="n">
-        <v>14.49</v>
+        <v>15.99</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>15.99</v>
       </c>
-      <c r="H68" s="3" t="n">
-        <v>10.4</v>
-      </c>
+      <c r="H68" s="3" t="n"/>
       <c r="I68" s="2" t="n">
-        <v>14.99</v>
+        <v>16.49</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>16.49</v>
@@ -25303,16 +25123,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
-        <v>57.96</v>
+        <v>62.49</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>62.49</v>
@@ -25347,16 +25165,14 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>43.99</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
-        <v>52.97</v>
+        <v>56.99</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>56.99</v>
@@ -25391,16 +25207,14 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
-        <v>52.97</v>
+        <v>56.49</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>56.49</v>
@@ -25435,14 +25249,12 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
@@ -25479,14 +25291,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
         <v>0</v>
       </c>
@@ -25523,14 +25333,12 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
         <v>0</v>
       </c>
@@ -25567,14 +25375,12 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H8" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
         <v>0</v>
       </c>
@@ -25611,14 +25417,12 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>45.99</v>
+        <v>48.99</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>48.99</v>
       </c>
-      <c r="H9" s="3" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
         <v>0</v>
       </c>
@@ -25655,14 +25459,12 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H10" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
         <v>0</v>
       </c>
@@ -25699,16 +25501,14 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H11" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H11" s="3" t="n"/>
       <c r="I11" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>80.98999999999999</v>
@@ -25739,16 +25539,14 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H12" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H12" s="3" t="n"/>
       <c r="I12" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>80.48999999999999</v>
@@ -25779,16 +25577,14 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H13" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>80.98999999999999</v>
@@ -25819,16 +25615,14 @@
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H14" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H14" s="3" t="n"/>
       <c r="I14" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>80.48999999999999</v>
@@ -25863,14 +25657,12 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>43.99</v>
       </c>
-      <c r="H15" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H15" s="3" t="n"/>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="n"/>
       <c r="K15" t="inlineStr">
@@ -25903,14 +25695,12 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H16" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="n"/>
       <c r="K16" t="inlineStr">
@@ -25943,14 +25733,12 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H17" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H17" s="3" t="n"/>
       <c r="I17" s="2" t="n">
         <v>0</v>
       </c>
@@ -25987,14 +25775,12 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H18" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
         <v>0</v>
       </c>
@@ -26031,14 +25817,12 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H19" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H19" s="3" t="n"/>
       <c r="I19" s="2" t="n">
         <v>0</v>
       </c>
@@ -26121,14 +25905,12 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H21" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H21" s="3" t="n"/>
       <c r="I21" s="2" t="n">
         <v>0</v>
       </c>
@@ -26165,14 +25947,12 @@
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H22" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H22" s="3" t="n"/>
       <c r="I22" s="2" t="n">
         <v>0</v>
       </c>
@@ -26209,14 +25989,12 @@
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H23" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H23" s="3" t="n"/>
       <c r="I23" s="2" t="n">
         <v>0</v>
       </c>
@@ -26253,14 +26031,12 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H24" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H24" s="3" t="n"/>
       <c r="I24" s="2" t="n">
         <v>0</v>
       </c>
@@ -26293,16 +26069,14 @@
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H25" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H25" s="3" t="n"/>
       <c r="I25" s="2" t="n">
-        <v>54.99</v>
+        <v>59.49</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>59.49</v>
@@ -26337,16 +26111,14 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>69.98999999999999</v>
+        <v>74.98999999999999</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>74.98999999999999</v>
       </c>
-      <c r="H26" s="3" t="n">
-        <v>7.1</v>
-      </c>
+      <c r="H26" s="3" t="n"/>
       <c r="I26" s="2" t="n">
-        <v>94.95999999999999</v>
+        <v>101.99</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>101.99</v>
@@ -26381,16 +26153,14 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H27" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H27" s="3" t="n"/>
       <c r="I27" s="2" t="n">
-        <v>74.98999999999999</v>
+        <v>80.48999999999999</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>80.48999999999999</v>
@@ -26425,16 +26195,14 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H28" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H28" s="3" t="n"/>
       <c r="I28" s="2" t="n">
-        <v>54.99</v>
+        <v>59.49</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>59.49</v>
@@ -26469,16 +26237,14 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H29" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H29" s="3" t="n"/>
       <c r="I29" s="2" t="n">
-        <v>54.99</v>
+        <v>59.49</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>59.49</v>
@@ -26597,16 +26363,14 @@
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
       <c r="F32" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H32" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H32" s="3" t="n"/>
       <c r="I32" s="2" t="n">
-        <v>49.49</v>
+        <v>52.99</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>52.99</v>
@@ -26637,16 +26401,14 @@
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" s="2" t="n">
-        <v>55.99</v>
+        <v>56.99</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>56.99</v>
       </c>
-      <c r="H33" s="3" t="n">
-        <v>1.8</v>
-      </c>
+      <c r="H33" s="3" t="n"/>
       <c r="I33" s="2" t="n">
-        <v>71.95</v>
+        <v>73.48999999999999</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>73.48999999999999</v>
@@ -26681,16 +26443,14 @@
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H34" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H34" s="3" t="n"/>
       <c r="I34" s="2" t="n">
-        <v>50.97</v>
+        <v>54.99</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>54.99</v>
@@ -26725,14 +26485,12 @@
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="n">
-        <v>39.99</v>
+        <v>42.99</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>42.99</v>
       </c>
-      <c r="H35" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H35" s="3" t="n"/>
       <c r="I35" s="2" t="n">
         <v>0</v>
       </c>
@@ -26769,16 +26527,14 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="n">
-        <v>59.99</v>
+        <v>63.99</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>63.99</v>
       </c>
-      <c r="H36" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H36" s="3" t="n"/>
       <c r="I36" s="2" t="n">
-        <v>80.95999999999999</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>86.48999999999999</v>
@@ -26813,16 +26569,14 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" s="2" t="n">
-        <v>44.99</v>
+        <v>47.99</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>47.99</v>
       </c>
-      <c r="H37" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H37" s="3" t="n"/>
       <c r="I37" s="2" t="n">
-        <v>56.96</v>
+        <v>60.99</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>60.99</v>
@@ -26857,14 +26611,12 @@
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" s="2" t="n">
-        <v>52.99</v>
+        <v>56.99</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>56.99</v>
       </c>
-      <c r="H38" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H38" s="3" t="n"/>
       <c r="I38" s="2" t="n">
         <v>0</v>
       </c>
@@ -26901,16 +26653,14 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H39" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H39" s="3" t="n"/>
       <c r="I39" s="2" t="n">
-        <v>64.95999999999999</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>69.98999999999999</v>
@@ -26941,16 +26691,14 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H40" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H40" s="3" t="n"/>
       <c r="I40" s="2" t="n">
-        <v>64.95999999999999</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>69.98999999999999</v>
@@ -26985,16 +26733,14 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H41" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H41" s="3" t="n"/>
       <c r="I41" s="2" t="n">
-        <v>61.26</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>65.98999999999999</v>
@@ -27025,16 +26771,14 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H42" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H42" s="3" t="n"/>
       <c r="I42" s="2" t="n">
-        <v>51.27</v>
+        <v>55.49</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>55.49</v>
@@ -27069,16 +26813,14 @@
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H43" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H43" s="3" t="n"/>
       <c r="I43" s="2" t="n">
-        <v>62.96</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>67.98999999999999</v>
@@ -27109,16 +26851,14 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
       <c r="F44" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H44" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H44" s="3" t="n"/>
       <c r="I44" s="2" t="n">
-        <v>62.96</v>
+        <v>67.98999999999999</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>67.98999999999999</v>
@@ -27149,16 +26889,14 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
       <c r="F45" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H45" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H45" s="3" t="n"/>
       <c r="I45" s="2" t="n">
-        <v>65.95</v>
+        <v>70.98999999999999</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>70.98999999999999</v>
@@ -27189,16 +26927,14 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H46" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H46" s="3" t="n"/>
       <c r="I46" s="2" t="n">
-        <v>55.97</v>
+        <v>60.49</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>60.49</v>
@@ -27233,16 +26969,14 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
       <c r="F47" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H47" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H47" s="3" t="n"/>
       <c r="I47" s="2" t="n">
-        <v>63.96</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>68.98999999999999</v>
@@ -27273,16 +27007,14 @@
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
       <c r="F48" s="2" t="n">
-        <v>49.99</v>
+        <v>53.99</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>53.99</v>
       </c>
-      <c r="H48" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="H48" s="3" t="n"/>
       <c r="I48" s="2" t="n">
-        <v>53.97</v>
+        <v>58.49</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>58.49</v>
@@ -27408,16 +27140,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>31.99</v>
+        <v>33.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>33.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>6.3</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
-        <v>34.99</v>
+        <v>36.99</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>36.99</v>
@@ -27452,16 +27182,14 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
-        <v>21.99</v>
+        <v>22.99</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>22.99</v>
@@ -27496,16 +27224,14 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
-        <v>21.99</v>
+        <v>22.99</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>22.99</v>
@@ -27678,14 +27404,12 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H8" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
         <v>0</v>
       </c>
@@ -27768,16 +27492,14 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>9.56</v>
+        <v>9.99</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>9.99</v>
       </c>
-      <c r="H10" s="3" t="n">
-        <v>4.5</v>
-      </c>
+      <c r="H10" s="3" t="n"/>
       <c r="I10" s="2" t="n">
-        <v>9.99</v>
+        <v>10.49</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>10.49</v>
@@ -27904,16 +27626,14 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>14.99</v>
+        <v>15.99</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>15.99</v>
       </c>
-      <c r="H13" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H13" s="3" t="n"/>
       <c r="I13" s="2" t="n">
-        <v>20.99</v>
+        <v>22.49</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>22.49</v>
@@ -28036,14 +27756,12 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>10.95</v>
+        <v>11.99</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H16" s="3" t="n">
-        <v>9.5</v>
-      </c>
+      <c r="H16" s="3" t="n"/>
       <c r="I16" s="2" t="n">
         <v>0</v>
       </c>
@@ -28080,14 +27798,12 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>10.95</v>
+        <v>11.99</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>11.99</v>
       </c>
-      <c r="H17" s="3" t="n">
-        <v>9.5</v>
-      </c>
+      <c r="H17" s="3" t="n"/>
       <c r="I17" s="2" t="n">
         <v>0</v>
       </c>
@@ -28124,14 +27840,12 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>28.99</v>
+        <v>30.99</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>30.99</v>
       </c>
-      <c r="H18" s="3" t="n">
-        <v>6.9</v>
-      </c>
+      <c r="H18" s="3" t="n"/>
       <c r="I18" s="2" t="n">
         <v>0</v>
       </c>
@@ -28168,14 +27882,12 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>9.56</v>
+        <v>9.99</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>9.99</v>
       </c>
-      <c r="H19" s="3" t="n">
-        <v>4.5</v>
-      </c>
+      <c r="H19" s="3" t="n"/>
       <c r="I19" s="2" t="n">
         <v>0</v>
       </c>
@@ -28212,14 +27924,12 @@
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>19.99</v>
+        <v>20.99</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>20.99</v>
       </c>
-      <c r="H20" s="3" t="n">
-        <v>5</v>
-      </c>
+      <c r="H20" s="3" t="n"/>
       <c r="I20" s="2" t="n">
         <v>0</v>
       </c>
@@ -28256,16 +27966,14 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>29.99</v>
+        <v>31.99</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>31.99</v>
       </c>
-      <c r="H21" s="3" t="n">
-        <v>6.7</v>
-      </c>
+      <c r="H21" s="3" t="n"/>
       <c r="I21" s="2" t="n">
-        <v>32.99</v>
+        <v>34.99</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>34.99</v>
@@ -29490,14 +29198,12 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
         <v>0</v>
       </c>
@@ -29534,14 +29240,12 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
         <v>0</v>
       </c>
@@ -29578,14 +29282,12 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
@@ -29622,14 +29324,12 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>130</v>
+        <v>139.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>139.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
         <v>0</v>
       </c>
@@ -29666,16 +29366,14 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>33.99</v>
+        <v>36.99</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>36.99</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>8.800000000000001</v>
-      </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
-        <v>35.99</v>
+        <v>38.99</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>38.99</v>
@@ -29756,16 +29454,14 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>119.99</v>
+        <v>128.99</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>128.99</v>
       </c>
-      <c r="H9" s="3" t="n">
-        <v>7.5</v>
-      </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>131.99</v>
+        <v>141.99</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>141.99</v>
@@ -30101,16 +29797,14 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
-        <v>55.99</v>
+        <v>59.99</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>59.99</v>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>7.1</v>
-      </c>
+      <c r="H2" s="3" t="n"/>
       <c r="I2" s="2" t="n">
-        <v>58.99</v>
+        <v>62.99</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>62.99</v>
@@ -30145,16 +29839,14 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
-        <v>33.99</v>
+        <v>34.99</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H3" s="3" t="n">
-        <v>2.9</v>
-      </c>
+      <c r="H3" s="3" t="n"/>
       <c r="I3" s="2" t="n">
-        <v>37.49</v>
+        <v>38.49</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>38.49</v>
@@ -30189,16 +29881,14 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
-        <v>63.99</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>68.98999999999999</v>
       </c>
-      <c r="H4" s="3" t="n">
-        <v>7.8</v>
-      </c>
+      <c r="H4" s="3" t="n"/>
       <c r="I4" s="2" t="n">
-        <v>70.48999999999999</v>
+        <v>75.98999999999999</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>75.98999999999999</v>
@@ -30233,16 +29923,14 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
-        <v>32.99</v>
+        <v>34.99</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>34.99</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>6.1</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="2" t="n">
-        <v>34.99</v>
+        <v>36.99</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>36.99</v>
@@ -30277,16 +29965,14 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>56.99</v>
+        <v>60.99</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>60.99</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>7</v>
-      </c>
+      <c r="H6" s="3" t="n"/>
       <c r="I6" s="2" t="n">
-        <v>62.49</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>66.98999999999999</v>
@@ -30321,16 +30007,14 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>40.99</v>
+        <v>43.99</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>43.99</v>
       </c>
-      <c r="H7" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H7" s="3" t="n"/>
       <c r="I7" s="2" t="n">
-        <v>42.99</v>
+        <v>45.99</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>45.99</v>
@@ -30365,16 +30049,14 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>41.99</v>
+        <v>44.99</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>44.99</v>
       </c>
-      <c r="H8" s="3" t="n">
-        <v>7.1</v>
-      </c>
+      <c r="H8" s="3" t="n"/>
       <c r="I8" s="2" t="n">
-        <v>43.99</v>
+        <v>46.99</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>46.99</v>
@@ -30409,16 +30091,14 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>54.99</v>
+        <v>58.99</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>58.99</v>
       </c>
-      <c r="H9" s="3" t="n">
-        <v>7.3</v>
-      </c>
+      <c r="H9" s="3" t="n"/>
       <c r="I9" s="2" t="n">
-        <v>73.95999999999999</v>
+        <v>79.48999999999999</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>79.48999999999999</v>

</xml_diff>